<commit_message>
second page and third page
</commit_message>
<xml_diff>
--- a/bd.xlsx
+++ b/bd.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\Python documents\Pere_kpoda\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\père kpoda\env\Pere_kpoda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D76C2CF-00F7-4265-9EBD-EEDD3878335D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="141">
   <si>
     <t>Date de dépôt</t>
   </si>
@@ -48,9 +47,6 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>Theme</t>
-  </si>
-  <si>
     <t>Thématique</t>
   </si>
   <si>
@@ -72,15 +68,9 @@
     <t>Mentions</t>
   </si>
   <si>
-    <t>Nitiema</t>
-  </si>
-  <si>
     <t>Wondpagnande Marceline</t>
   </si>
   <si>
-    <t>Nitiema Wondpagnande Marceline</t>
-  </si>
-  <si>
     <t>Mise en place d'une comptablité générale dans les EPN: cas de l'EPN Alpha</t>
   </si>
   <si>
@@ -96,15 +86,9 @@
     <t>Très Bien</t>
   </si>
   <si>
-    <t>Evilaro</t>
-  </si>
-  <si>
     <t>Grâce Ursula Aye</t>
   </si>
   <si>
-    <t>Evilaro Grâce Ursula Aye</t>
-  </si>
-  <si>
     <t>Audit interne dans la performance finiancère d'une compagnie d'assurance: SIDAM-CI S.A</t>
   </si>
   <si>
@@ -192,9 +176,6 @@
     <t>Kouassi Yves Herman</t>
   </si>
   <si>
-    <t>Analalyse de l'impact de l'extension du reseau de soins de NSIA ASSURANCES sur les prestations commerciales</t>
-  </si>
-  <si>
     <t>Assurance</t>
   </si>
   <si>
@@ -202,12 +183,282 @@
   </si>
   <si>
     <t>NSIA ASSURANCES</t>
+  </si>
+  <si>
+    <t>DRABO</t>
+  </si>
+  <si>
+    <t>Fatoumata</t>
+  </si>
+  <si>
+    <t>DRAGO Fatoumata</t>
+  </si>
+  <si>
+    <t>Analyse de l'impact de l'extension du reseau de soins de NSIA ASSURANCES sur les prestations commerciales</t>
+  </si>
+  <si>
+    <t>NITIEMA Wondpagnande Marceline</t>
+  </si>
+  <si>
+    <t>NITIEMA</t>
+  </si>
+  <si>
+    <t>EVILARO</t>
+  </si>
+  <si>
+    <t>EVILARO Grâce Ursula Aye</t>
+  </si>
+  <si>
+    <t>Analyse de la politique de vente du produit financier "performa" de la loyale vie</t>
+  </si>
+  <si>
+    <t>loyale vie</t>
+  </si>
+  <si>
+    <t>OSSEY</t>
+  </si>
+  <si>
+    <t>Kopoin Jean Martial. E</t>
+  </si>
+  <si>
+    <t>OSSEY Kopoin Jean Martial</t>
+  </si>
+  <si>
+    <t>Financement des PME à la SIB analyse des difficultés d'accès</t>
+  </si>
+  <si>
+    <t>Banque</t>
+  </si>
+  <si>
+    <t>SIB</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-05-11 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-05-07 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-01-05 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-02-09 00:00:00</t>
+  </si>
+  <si>
+    <t>KDEA</t>
+  </si>
+  <si>
+    <t>Esther Marie-Noelle</t>
+  </si>
+  <si>
+    <t>KDEA Esther Marie-Noelle</t>
+  </si>
+  <si>
+    <t>Effet de la consommation des énergies renouvelables sur la croissance économique</t>
+  </si>
+  <si>
+    <t>Economie du développement</t>
+  </si>
+  <si>
+    <t>Thème</t>
+  </si>
+  <si>
+    <t>FOFANA</t>
+  </si>
+  <si>
+    <t>Bala Fatim Georgia</t>
+  </si>
+  <si>
+    <t>KANGA</t>
+  </si>
+  <si>
+    <t>Ange Leandre</t>
+  </si>
+  <si>
+    <t>Analyse de la chaîne de valeur du manioc dans la région du GBÈKÈ EN Côte d'Ivoire : exemple de la scoop-ca</t>
+  </si>
+  <si>
+    <t>Analyse de la gestion de la relation client dans le milieu bancaire : cas de la SGCI</t>
+  </si>
+  <si>
+    <t>Gnanzou Michel-Emmanuel</t>
+  </si>
+  <si>
+    <t>Evaluation de la procédure d'inventaire au bureau national d'études techniques</t>
+  </si>
+  <si>
+    <t>TRAORE</t>
+  </si>
+  <si>
+    <t>Hadja Nissia</t>
+  </si>
+  <si>
+    <t>Analyse des facteurs des impayés dans une institution de microfinance : cas de Credit Access</t>
+  </si>
+  <si>
+    <t>KANGA Ange Leandre</t>
+  </si>
+  <si>
+    <t>KOUAME Gnanzou Michel-Emmanuel</t>
+  </si>
+  <si>
+    <t>FOFANA Bala Fatim Georgia</t>
+  </si>
+  <si>
+    <t>TRAORE Hadja Nissia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-03-31 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-03-15 00:00:00</t>
+  </si>
+  <si>
+    <t>scoop-ca</t>
+  </si>
+  <si>
+    <t>Credit Access</t>
+  </si>
+  <si>
+    <t>SGCI</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-05-06 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-05-18 00:00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2021-05-14 00:00:00</t>
+  </si>
+  <si>
+    <t>les énergies renouvelables</t>
+  </si>
+  <si>
+    <t>développement durable</t>
+  </si>
+  <si>
+    <t>epsilon</t>
+  </si>
+  <si>
+    <t>ALPHA</t>
+  </si>
+  <si>
+    <t>EPN Alpha</t>
+  </si>
+  <si>
+    <t>KOFFI</t>
+  </si>
+  <si>
+    <t>Ahou Marie Madelaine</t>
+  </si>
+  <si>
+    <t>OUATTARA</t>
+  </si>
+  <si>
+    <t>Abdul Aziz</t>
+  </si>
+  <si>
+    <t>BAYALA</t>
+  </si>
+  <si>
+    <t>Epio Odette</t>
+  </si>
+  <si>
+    <t>Optimisation du risque de crédit liée à la clientèle professionnelle : cas de la banque populaire de Côte d'Ivoire</t>
+  </si>
+  <si>
+    <t>Analyse du système de gestion pour l'assurance IARDT : cas de la banque Atlantique de Côte d'Ivoire</t>
+  </si>
+  <si>
+    <t>Disparité départementales de pauvreté en Côte d'Ivoire : une analyse à partir de l'économétrie spatiale</t>
+  </si>
+  <si>
+    <t>banque populaire</t>
+  </si>
+  <si>
+    <t>banque Atlantique</t>
+  </si>
+  <si>
+    <t>MEL</t>
+  </si>
+  <si>
+    <t>Orlane Valesca</t>
+  </si>
+  <si>
+    <t>Marc Yvan</t>
+  </si>
+  <si>
+    <t>YAO</t>
+  </si>
+  <si>
+    <t>ELUH</t>
+  </si>
+  <si>
+    <t>Affoué Sarah Stéphanie</t>
+  </si>
+  <si>
+    <t>Ayikoé Théophilus</t>
+  </si>
+  <si>
+    <t>ADANLETE</t>
+  </si>
+  <si>
+    <t>Evaluation de la pratique du crédit bail sur le marché des particuliers : cas de la BICICI</t>
+  </si>
+  <si>
+    <t>Analyse du reseau d'agence et ses performances commerciales : cas de la Banque Populaire de Côte d'Ivoire</t>
+  </si>
+  <si>
+    <t>Analyse de la gestion du risque inhérent à l'octroi de crédit bancaire aux entreprises : cas d'Afriland First Bank</t>
+  </si>
+  <si>
+    <t>Mise en place d'un manuel de procédures du cycle ventes-clients d'une société commerciale : cas de la société GEDI.MAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2021-05-14 00:00:00</t>
+  </si>
+  <si>
+    <t>BICICI</t>
+  </si>
+  <si>
+    <t>Afriland First Bank</t>
+  </si>
+  <si>
+    <t>GEDI.MAT</t>
+  </si>
+  <si>
+    <t>KOFFI Ahou Marie Madelaine</t>
+  </si>
+  <si>
+    <t>OUATTARA Abdul Aziz</t>
+  </si>
+  <si>
+    <t>BAYALA Epio Odette</t>
+  </si>
+  <si>
+    <t>MEL Orlane Valesca</t>
+  </si>
+  <si>
+    <t>YAO Marc Yvan</t>
+  </si>
+  <si>
+    <t>ELUH Affoué Sarah Stéphanie</t>
+  </si>
+  <si>
+    <t>ADANLETE Ayikoé Théophilus</t>
+  </si>
+  <si>
+    <t>Pauvreté</t>
+  </si>
+  <si>
+    <t>gestion de risque</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
@@ -260,12 +511,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,23 +831,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Feuil1"/>
+  <dimension ref="A1:M23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="101.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="102.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.6328125" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -600,299 +867,789 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>44123</v>
       </c>
       <c r="B2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
+        <v>104</v>
+      </c>
+      <c r="L2" s="6">
+        <v>44146</v>
+      </c>
+      <c r="M2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" s="2">
-        <v>44146</v>
-      </c>
-      <c r="M2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>44123</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="L3" s="6">
+        <v>44146</v>
+      </c>
+      <c r="M3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" s="2">
-        <v>44146</v>
-      </c>
-      <c r="M3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>44120</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="s">
         <v>28</v>
       </c>
-      <c r="C4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="2">
+      <c r="L4" s="6">
         <v>44187</v>
       </c>
       <c r="M4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>44120</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L5" s="2">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>102</v>
+      </c>
+      <c r="L5" s="6">
         <v>44187</v>
       </c>
       <c r="M5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>44166</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
         <v>41</v>
       </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" t="s">
-        <v>46</v>
-      </c>
-      <c r="L6" s="2">
+      <c r="L6" s="6">
         <v>44186</v>
       </c>
       <c r="M6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>44167</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="I7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L7" s="2">
+        <v>16</v>
+      </c>
+      <c r="J7" t="s">
+        <v>103</v>
+      </c>
+      <c r="L7" s="6">
         <v>44187</v>
       </c>
       <c r="M7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>44167</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
-      </c>
-      <c r="L8" s="2">
+        <v>46</v>
+      </c>
+      <c r="L8" s="6">
         <v>44187</v>
       </c>
       <c r="M8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>44167</v>
       </c>
       <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
         <v>47</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9" t="s">
+        <v>50</v>
+      </c>
+      <c r="L9" s="6">
+        <v>44186</v>
+      </c>
+      <c r="M9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
         <v>52</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" t="s">
         <v>49</v>
       </c>
-      <c r="F9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" t="s">
-        <v>54</v>
-      </c>
-      <c r="I9" t="s">
-        <v>55</v>
-      </c>
-      <c r="J9" t="s">
-        <v>56</v>
-      </c>
-      <c r="L9" s="2">
-        <v>44186</v>
-      </c>
-      <c r="M9" t="s">
+      <c r="J10" t="s">
+        <v>60</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="M10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" t="s">
+        <v>49</v>
+      </c>
+      <c r="J11" t="s">
+        <v>66</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="M11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" t="s">
+        <v>101</v>
+      </c>
+      <c r="I12" t="s">
+        <v>75</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="M12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" t="s">
+        <v>90</v>
+      </c>
+      <c r="F13" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" t="s">
+        <v>94</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="M13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" t="s">
+        <v>65</v>
+      </c>
+      <c r="I14" t="s">
+        <v>49</v>
+      </c>
+      <c r="J14" t="s">
+        <v>96</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="M14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" t="s">
+        <v>89</v>
+      </c>
+      <c r="F15" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" t="s">
         <v>27</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="M15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" t="s">
+        <v>65</v>
+      </c>
+      <c r="I16" t="s">
+        <v>49</v>
+      </c>
+      <c r="J16" t="s">
+        <v>95</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="M16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" t="s">
+        <v>111</v>
+      </c>
+      <c r="G17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H17" t="s">
+        <v>65</v>
+      </c>
+      <c r="I17" t="s">
+        <v>49</v>
+      </c>
+      <c r="J17" t="s">
+        <v>114</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="M17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" t="s">
+        <v>112</v>
+      </c>
+      <c r="G18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18" t="s">
+        <v>48</v>
+      </c>
+      <c r="I18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" t="s">
+        <v>134</v>
+      </c>
+      <c r="F19" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" t="s">
+        <v>139</v>
+      </c>
+      <c r="H19" t="s">
+        <v>75</v>
+      </c>
+      <c r="I19" t="s">
+        <v>75</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="M19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" t="s">
+        <v>135</v>
+      </c>
+      <c r="F20" t="s">
+        <v>124</v>
+      </c>
+      <c r="G20" t="s">
+        <v>65</v>
+      </c>
+      <c r="H20" t="s">
+        <v>65</v>
+      </c>
+      <c r="I20" t="s">
+        <v>49</v>
+      </c>
+      <c r="J20" t="s">
+        <v>129</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" t="s">
+        <v>136</v>
+      </c>
+      <c r="F21" t="s">
+        <v>125</v>
+      </c>
+      <c r="G21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" t="s">
+        <v>65</v>
+      </c>
+      <c r="I21" t="s">
+        <v>49</v>
+      </c>
+      <c r="J21" t="s">
+        <v>114</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="M21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" t="s">
+        <v>121</v>
+      </c>
+      <c r="D22" t="s">
+        <v>137</v>
+      </c>
+      <c r="F22" t="s">
+        <v>126</v>
+      </c>
+      <c r="G22" t="s">
+        <v>140</v>
+      </c>
+      <c r="H22" t="s">
+        <v>65</v>
+      </c>
+      <c r="I22" t="s">
+        <v>49</v>
+      </c>
+      <c r="J22" t="s">
+        <v>130</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>92</v>
+      </c>
+      <c r="B23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" t="s">
+        <v>122</v>
+      </c>
+      <c r="D23" t="s">
+        <v>138</v>
+      </c>
+      <c r="F23" t="s">
+        <v>127</v>
+      </c>
+      <c r="G23" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" t="s">
+        <v>16</v>
+      </c>
+      <c r="J23" t="s">
+        <v>131</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="M23" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>